<commit_message>
migrated codebase to object orientated
started using uv
</commit_message>
<xml_diff>
--- a/example/example/example_HouseBlend_period_1_mailmerge.xlsx
+++ b/example/example/example_HouseBlend_period_1_mailmerge.xlsx
@@ -484,312 +484,312 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>John Pennington</t>
+          <t>Wesley Gray</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>John</t>
+          <t>Wesley</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>John Pennington</t>
+          <t>Wesley Gray</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Melissa Hernandez</t>
+          <t>Lauren Williams</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Melissa</t>
+          <t>Lauren</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>01/03/2026</t>
+          <t>08/03/2026</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>15/03/2026</t>
+          <t>22/03/2026</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Sunday 1st March 2026</t>
+          <t>Sunday 8th March 2026</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Sunday 15th March 2026</t>
+          <t>Sunday 22nd March 2026</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>JohnPennington@email.com</t>
+          <t>WesleyGray@email.com</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Melissa Hernandez</t>
+          <t>Lauren Williams</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Melissa</t>
+          <t>Lauren</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Melissa Hernandez</t>
+          <t>Lauren Williams</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>John Pennington</t>
+          <t>Wesley Gray</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>John</t>
+          <t>Wesley</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>01/03/2026</t>
+          <t>08/03/2026</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>15/03/2026</t>
+          <t>22/03/2026</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Sunday 1st March 2026</t>
+          <t>Sunday 8th March 2026</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Sunday 15th March 2026</t>
+          <t>Sunday 22nd March 2026</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>MelissaHernandez@email.com</t>
+          <t>LaurenWilliams@email.com</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Joshua Sloan</t>
+          <t>Allison Harris</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Joshua</t>
+          <t>Allison</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Joshua Sloan</t>
+          <t>Allison Harris</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Crystal Figueroa</t>
+          <t>Amber Lawson</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Crystal</t>
+          <t>Amber</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>01/03/2026</t>
+          <t>08/03/2026</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>15/03/2026</t>
+          <t>22/03/2026</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Sunday 1st March 2026</t>
+          <t>Sunday 8th March 2026</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Sunday 15th March 2026</t>
+          <t>Sunday 22nd March 2026</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>JoshuaSloan@email.com</t>
+          <t>AllisonHarris@email.com</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Crystal Figueroa</t>
+          <t>Amber Lawson</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Crystal</t>
+          <t>Amber</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Crystal Figueroa</t>
+          <t>Amber Lawson</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Joshua Sloan</t>
+          <t>Allison Harris</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Joshua</t>
+          <t>Allison</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>01/03/2026</t>
+          <t>08/03/2026</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>15/03/2026</t>
+          <t>22/03/2026</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Sunday 1st March 2026</t>
+          <t>Sunday 8th March 2026</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Sunday 15th March 2026</t>
+          <t>Sunday 22nd March 2026</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>CrystalFigueroa@email.com</t>
+          <t>AmberLawson@email.com</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>William Sims</t>
+          <t>Beverly Clark</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>William</t>
+          <t>Beverly</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>William Sims</t>
+          <t>Beverly Clark</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Kevin Munoz</t>
+          <t>Gabriel Arnold</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Kevin</t>
+          <t>Gabriel</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>01/03/2026</t>
+          <t>08/03/2026</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>15/03/2026</t>
+          <t>22/03/2026</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Sunday 1st March 2026</t>
+          <t>Sunday 8th March 2026</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Sunday 15th March 2026</t>
+          <t>Sunday 22nd March 2026</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>WilliamSims@email.com</t>
+          <t>BeverlyClark@email.com</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Kevin Munoz</t>
+          <t>Gabriel Arnold</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Kevin</t>
+          <t>Gabriel</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Kevin Munoz</t>
+          <t>Gabriel Arnold</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>William Sims</t>
+          <t>Beverly Clark</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>William</t>
+          <t>Beverly</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>01/03/2026</t>
+          <t>08/03/2026</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>15/03/2026</t>
+          <t>22/03/2026</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Sunday 1st March 2026</t>
+          <t>Sunday 8th March 2026</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Sunday 15th March 2026</t>
+          <t>Sunday 22nd March 2026</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>KevinMunoz@email.com</t>
+          <t>GabrielArnold@email.com</t>
         </is>
       </c>
     </row>
@@ -867,342 +867,342 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>John Pennington</t>
+          <t>Wesley Gray</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>John</t>
+          <t>Wesley</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>John Pennington</t>
+          <t>Wesley Gray</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Melissa Hernandez</t>
+          <t>Lauren Williams</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Melissa Hernandez</t>
+          <t>Lauren Williams</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>MelissaHernandez@email.com</t>
+          <t>LaurenWilliams@email.com</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>01/03/2026</t>
+          <t>08/03/2026</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>15/03/2026</t>
+          <t>22/03/2026</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Sunday 1st March 2026</t>
+          <t>Sunday 8th March 2026</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Sunday 15th March 2026</t>
+          <t>Sunday 22nd March 2026</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>JohnPennington@email.com</t>
+          <t>WesleyGray@email.com</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Melissa Hernandez</t>
+          <t>Lauren Williams</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Melissa</t>
+          <t>Lauren</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Melissa Hernandez</t>
+          <t>Lauren Williams</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>John Pennington</t>
+          <t>Wesley Gray</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>John Pennington</t>
+          <t>Wesley Gray</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>JohnPennington@email.com</t>
+          <t>WesleyGray@email.com</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>01/03/2026</t>
+          <t>08/03/2026</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>15/03/2026</t>
+          <t>22/03/2026</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Sunday 1st March 2026</t>
+          <t>Sunday 8th March 2026</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Sunday 15th March 2026</t>
+          <t>Sunday 22nd March 2026</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>MelissaHernandez@email.com</t>
+          <t>LaurenWilliams@email.com</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Joshua Sloan</t>
+          <t>Allison Harris</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Joshua</t>
+          <t>Allison</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Joshua Sloan</t>
+          <t>Allison Harris</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Crystal Figueroa</t>
+          <t>Amber Lawson</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Crystal Figueroa</t>
+          <t>Amber Lawson</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>CrystalFigueroa@email.com</t>
+          <t>AmberLawson@email.com</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>01/03/2026</t>
+          <t>08/03/2026</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>15/03/2026</t>
+          <t>22/03/2026</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Sunday 1st March 2026</t>
+          <t>Sunday 8th March 2026</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Sunday 15th March 2026</t>
+          <t>Sunday 22nd March 2026</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>JoshuaSloan@email.com</t>
+          <t>AllisonHarris@email.com</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Crystal Figueroa</t>
+          <t>Amber Lawson</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Crystal</t>
+          <t>Amber</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Crystal Figueroa</t>
+          <t>Amber Lawson</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Joshua Sloan</t>
+          <t>Allison Harris</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Joshua Sloan</t>
+          <t>Allison Harris</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>JoshuaSloan@email.com</t>
+          <t>AllisonHarris@email.com</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>01/03/2026</t>
+          <t>08/03/2026</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>15/03/2026</t>
+          <t>22/03/2026</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Sunday 1st March 2026</t>
+          <t>Sunday 8th March 2026</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Sunday 15th March 2026</t>
+          <t>Sunday 22nd March 2026</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>CrystalFigueroa@email.com</t>
+          <t>AmberLawson@email.com</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>William Sims</t>
+          <t>Beverly Clark</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>William</t>
+          <t>Beverly</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>William Sims</t>
+          <t>Beverly Clark</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Kevin Munoz</t>
+          <t>Gabriel Arnold</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Kevin Munoz</t>
+          <t>Gabriel Arnold</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>KevinMunoz@email.com</t>
+          <t>GabrielArnold@email.com</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>01/03/2026</t>
+          <t>08/03/2026</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>15/03/2026</t>
+          <t>22/03/2026</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Sunday 1st March 2026</t>
+          <t>Sunday 8th March 2026</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Sunday 15th March 2026</t>
+          <t>Sunday 22nd March 2026</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>WilliamSims@email.com</t>
+          <t>BeverlyClark@email.com</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Kevin Munoz</t>
+          <t>Gabriel Arnold</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Kevin</t>
+          <t>Gabriel</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Kevin Munoz</t>
+          <t>Gabriel Arnold</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>William Sims</t>
+          <t>Beverly Clark</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>William Sims</t>
+          <t>Beverly Clark</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>WilliamSims@email.com</t>
+          <t>BeverlyClark@email.com</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>01/03/2026</t>
+          <t>08/03/2026</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>15/03/2026</t>
+          <t>22/03/2026</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Sunday 1st March 2026</t>
+          <t>Sunday 8th March 2026</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Sunday 15th March 2026</t>
+          <t>Sunday 22nd March 2026</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>KevinMunoz@email.com</t>
+          <t>GabrielArnold@email.com</t>
         </is>
       </c>
     </row>

</xml_diff>